<commit_message>
lit review 11 papers completed
</commit_message>
<xml_diff>
--- a/papers/papers_tracker.xlsx
+++ b/papers/papers_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1abdca93598a4eb/Documents/SP Jain/3. Year 3/Semester 6/2. Computer Vision/Group Project/NeurIPS/vlm-radiology-report-gen/papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="8_{E925B9B9-A7FE-46D2-8C81-8C867BCA288A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0E355C1-D9DF-4557-A9C8-1CCD21A3E571}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{E925B9B9-A7FE-46D2-8C81-8C867BCA288A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F5F02BB-EA55-4782-A997-672D0BB8E12D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{15661808-99BE-4653-9C47-D65197835AC1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>Title</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>https://aclanthology.org/2022.emnlp-main.256/</t>
+  </si>
+  <si>
+    <t>Recent Progress in Deep Learning for Chest X-Ray Report Generation</t>
+  </si>
+  <si>
+    <t>Mounir Salhi, Moulay A. Akhloufi</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/publication/399620527_Recent_Progress_in_Deep_Learning_for_Chest_X-Ray_Report_Generation</t>
   </si>
 </sst>
 </file>
@@ -854,15 +863,23 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="6"/>
       <c r="E14" s="7"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="7"/>
+      <c r="H14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>

</xml_diff>

<commit_message>
added 18 papers lit review
</commit_message>
<xml_diff>
--- a/papers/papers_tracker.xlsx
+++ b/papers/papers_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1abdca93598a4eb/Documents/SP Jain/3. Year 3/Semester 6/2. Computer Vision/Group Project/NeurIPS/vlm-radiology-report-gen/papers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{E925B9B9-A7FE-46D2-8C81-8C867BCA288A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F5F02BB-EA55-4782-A997-672D0BB8E12D}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{E925B9B9-A7FE-46D2-8C81-8C867BCA288A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18994C93-1870-4790-AF66-54F7D453E21B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{15661808-99BE-4653-9C47-D65197835AC1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="93">
   <si>
     <t>Title</t>
   </si>
@@ -168,6 +168,171 @@
   </si>
   <si>
     <t>https://www.researchgate.net/publication/399620527_Recent_Progress_in_Deep_Learning_for_Chest_X-Ray_Report_Generation</t>
+  </si>
+  <si>
+    <t>Learning Transferable Visual Models From Natural Language Supervision</t>
+  </si>
+  <si>
+    <t>Alec Radford, Jong Wook Kim, Chris Hallacy, Aditya Ramesh, Gabriel Goh, Sandhini Agarwal, Girish Sastry, Amanda Askell, Pamela Mishkin, Jack Clark, Gretchen Krueger, Ilya Sutskever</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2103.00020</t>
+  </si>
+  <si>
+    <t>MediVLM: A Vision Language Model for Radiology Report Generation from Medical Images</t>
+  </si>
+  <si>
+    <t>Debanjan Goswami, Ronast Subedi, Shayok Chakraborty</t>
+  </si>
+  <si>
+    <t>https://aclanthology.org/2025.findings-emnlp.544/</t>
+  </si>
+  <si>
+    <t>Dasith Edirisinghe; Wimukthi Nimalsiri; Mahela Hennayake; Dulani Meedeniya; Gilbert Lim</t>
+  </si>
+  <si>
+    <t>Chest X-Ray Report Generation Using Abnormality Guided Vision Language Model</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/11153468</t>
+  </si>
+  <si>
+    <t>Suppressing Prior-Comparison Hallucinations in Radiology Report Generation via Semantically Decoupled Latent Steering</t>
+  </si>
+  <si>
+    <t>Ao Li, Rui Liu, Mingjie Li, Sheng Liu, Lei Wang, Xiaodan Liang, Lina Yao, Xiaojun Chang, Lei Xing</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2602.23676</t>
+  </si>
+  <si>
+    <t>FactCheXcker: Mitigating Measurement Hallucinations in Chest X-ray Report Generation Models</t>
+  </si>
+  <si>
+    <t>Alice Heiman, Xiaoman Zhang, Emma Chen, Sung Eun Kim, Pranav Rajpurkar</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2411.18672</t>
+  </si>
+  <si>
+    <t>Collaboration between clinicians and vision–language models in radiology report generation</t>
+  </si>
+  <si>
+    <t>Ryutaro Tanno, David G. T. Barrett, Andrew Sellergren, Sumedh Ghaisas, Sumanth Dathathri, Abigail See, Johannes Welbl, Charles Lau, Tao Tu, Shekoofeh Azizi, Karan Singhal, Mike Schaekermann, Rhys May, Roy Lee, SiWai Man, Sara Mahdavi, Zahra Ahmed, Yossi Matias, Joelle Barral, S. M. Ali Eslami, Danielle Belgrave, Yun Liu, Sreenivasa Raju Kalidindi, Shravya Shetty, Vivek Natarajan, Pushmeet Kohli, Po-Sen Huang, Alan Karthikesalingam &amp; Ira Ktena</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41591-024-03302-1</t>
+  </si>
+  <si>
+    <t>Automatic Radiology Report Generation: A Comprehensive Review and Innovative Framework</t>
+  </si>
+  <si>
+    <t>Moustapha Boubacar Hamma
+LIASSE LAB, ENSA-Sidi Mohamed Ben Abdallah University of Fez, Morocco
+; Zakariae Alami Merrouni; Bouchra Frikh; Brahim Ouhbi</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/10821974</t>
+  </si>
+  <si>
+    <t>Show, Attend and Tell: Neural Image Caption Generation with Visual Attention</t>
+  </si>
+  <si>
+    <t>Kelvin Xu, Jimmy Ba, Ryan Kiros, Kyunghyun Cho, Aaron Courville, Ruslan Salakhutdinov, Richard Zemel, Yoshua Bengio</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/1502.03044</t>
+  </si>
+  <si>
+    <t>Making the Most of Text Semantics to Improve Biomedical Vision--Language Processing</t>
+  </si>
+  <si>
+    <t>Benedikt Boecking, Naoto Usuyama, Shruthi Bannur, Daniel C. Castro, Anton Schwaighofer, Stephanie Hyland, Maria Wetscherek, Tristan Naumann, Aditya Nori, Javier Alvarez-Valle, Hoifung Poon, Ozan Oktay</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2204.09817</t>
+  </si>
+  <si>
+    <t>Evaluating progress in automatic chest X-ray radiology report generation</t>
+  </si>
+  <si>
+    <t>Feiyang Yu, Mark Endo, Rayan Krishnan, Ian Pan, Andy Tsai, Eduardo Pontes Reis, Eduardo Kaiser Ururahy Nunes Fonseca, Henrique Min Ho Lee, Zahra Shakeri Hossein Abad, Andrew Y Ng, Curtis P Langlotz, Vasantha Kumar Venugopal, Pranav Rajpurkar</t>
+  </si>
+  <si>
+    <t>https://pubmed.ncbi.nlm.nih.gov/37720336/</t>
+  </si>
+  <si>
+    <t>BERTScore: Evaluating Text Generation with BERT</t>
+  </si>
+  <si>
+    <t>Tianyi Zhang, Varsha Kishore, Felix Wu, Kilian Q. Weinberger, Yoav Artzi</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/1904.09675</t>
+  </si>
+  <si>
+    <t>Preparing a collection of radiology examinations for distribution and retrieval</t>
+  </si>
+  <si>
+    <t>Dina Demner-Fushman, Marc D Kohli, Marc B Rosenman, Sonya E Shooshan, Laritza Rodriguez, Sameer Antani, George R Thoma, Clement J McDonald</t>
+  </si>
+  <si>
+    <t>https://pubmed.ncbi.nlm.nih.gov/26133894/</t>
+  </si>
+  <si>
+    <t>Interactive and Explainable Region-guided Radiology Report Generation</t>
+  </si>
+  <si>
+    <t>Tim Tanida, Philip Müller, Georgios Kaissis, Daniel Rueckert</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2304.08295</t>
+  </si>
+  <si>
+    <t>RaDialog: A Large Vision-Language Model for Radiology Report Generation and Conversational Assistance</t>
+  </si>
+  <si>
+    <t>Chantal Pellegrini, Ege Özsoy, Benjamin Busam, Nassir Navab, Matthias Keicher</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2311.18681</t>
+  </si>
+  <si>
+    <t>CheXpert: A Large Chest Radiograph Dataset with Uncertainty Labels and Expert Comparison</t>
+  </si>
+  <si>
+    <t>Jeremy Irvin, Pranav Rajpurkar, Michael Ko, Yifan Yu, Silviana Ciurea-Ilcus, Chris Chute, Henrik Marklund, Behzad Haghgoo, Robyn Ball, Katie Shpanskaya, Jayne Seekins, David A. Mong, Safwan S. Halabi, Jesse K. Sandberg, Ricky Jones, David B. Larson, Curtis P. Langlotz, Bhavik N. Patel, Matthew P. Lungren, Andrew Y. Ng</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/1901.07031</t>
+  </si>
+  <si>
+    <t>Act Like a Radiologist: Radiology Report Generation
+Across Anatomical Regions</t>
+  </si>
+  <si>
+    <t>Qi Chen, Yutong Xie, Biao Wu, Xiaomin Chen, James Ang, Minh-Son To, Xiaojun Chang, Qi Wu</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2305.16685</t>
+  </si>
+  <si>
+    <t>HistGen: Histopathology Report Generation via Local-Global Feature Encoding and Cross-modal Context Interaction</t>
+  </si>
+  <si>
+    <t>Zhengrui Guo, Jiabo Ma, Yingxue Xu, Yihui Wang, Liansheng Wang, Hao Chen</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2403.05396</t>
+  </si>
+  <si>
+    <t>Hallucination Mitigating for Medical Report Generation</t>
+  </si>
+  <si>
+    <t>Ruoqing Zhao, Runze Xia, Piji Li</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2601.15745</t>
   </si>
 </sst>
 </file>
@@ -901,185 +1066,329 @@
       <c r="J16" s="6"/>
       <c r="K16" s="7"/>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="6"/>
       <c r="E17" s="7"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J17" s="6">
+        <v>2021</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="72" x14ac:dyDescent="0.3">
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="6"/>
       <c r="E18" s="7"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="J18" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="72" x14ac:dyDescent="0.3">
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="6"/>
       <c r="E19" s="7"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J19" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="6"/>
       <c r="E20" s="7"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H20" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="6"/>
       <c r="E21" s="7"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J21" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="316.8" x14ac:dyDescent="0.3">
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="6"/>
       <c r="E22" s="7"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="7"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H22" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J22" s="6">
+        <v>2024</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="6"/>
       <c r="E23" s="7"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="7"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H23" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J23" s="6">
+        <v>2024</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="6"/>
       <c r="E24" s="7"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="7"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H24" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="J24" s="6">
+        <v>2015</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="6"/>
       <c r="E25" s="7"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="7"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H25" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="J25" s="6">
+        <v>2022</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="6"/>
       <c r="E26" s="7"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="7"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H26" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J26" s="6">
+        <v>2023</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="6"/>
       <c r="E27" s="7"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="7"/>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H27" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J27" s="6">
+        <v>2019</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="6"/>
       <c r="E28" s="7"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="7"/>
-    </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H28" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J28" s="6">
+        <v>2016</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="6"/>
       <c r="E29" s="7"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="6"/>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H29" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J29" s="6">
+        <v>2023</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="6"/>
       <c r="E30" s="7"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="7"/>
-    </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H30" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J30" s="6">
+        <v>2025</v>
+      </c>
+      <c r="K30" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" ht="201.6" x14ac:dyDescent="0.3">
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="6"/>
       <c r="E31" s="7"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="7"/>
-    </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J31" s="6">
+        <v>2019</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
       <c r="D32" s="6"/>
       <c r="E32" s="7"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="7"/>
-    </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H32" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J32" s="6">
+        <v>2023</v>
+      </c>
+      <c r="K32" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
       <c r="D33" s="6"/>
       <c r="E33" s="7"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="7"/>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H33" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="J33" s="6">
+        <v>2024</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
       <c r="E34" s="7"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="7"/>
+      <c r="H34" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J34" s="6">
+        <v>2026</v>
+      </c>
+      <c r="K34" s="7" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B35" s="5"/>
@@ -8406,6 +8715,9 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K4" r:id="rId1" xr:uid="{EB68AF17-78E5-4525-97E9-12A8A1E2D154}"/>
+    <hyperlink ref="K22" r:id="rId2" xr:uid="{AF6EE124-BBB0-48C1-B832-2123A1227B16}"/>
+    <hyperlink ref="K29" r:id="rId3" xr:uid="{DD473016-74E6-47A2-8560-1C739AD95F0F}"/>
+    <hyperlink ref="K32" r:id="rId4" xr:uid="{507E3F81-D60F-4A7C-ACBA-27B3A2FA2A74}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>